<commit_message>
updated PNY SSD files to include DiskDrill and PhotoRec recovery data
</commit_message>
<xml_diff>
--- a/SSD Files/PNY CS900/Secure Erase/Recovery metrics.xlsx
+++ b/SSD Files/PNY CS900/Secure Erase/Recovery metrics.xlsx
@@ -5,15 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\Uni\Dissertation\MScProject\SSD Files\Kingston A400\Secure Erase\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\Uni\Dissertation\SSD Files\PNY CS900\Secure Erase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBAB18EA-C036-42ED-9C8E-547EDD22C684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A7E609-08FB-44DB-A69D-48B4481B6824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4720C983-EA5C-4C7A-96E6-6ACFA6986950}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Autopsy" sheetId="1" r:id="rId1"/>
+    <sheet name="DiskDrill" sheetId="2" r:id="rId2"/>
+    <sheet name="PhotoRec" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
   <si>
     <t>Volume</t>
   </si>
@@ -60,13 +62,34 @@
     <t>Scenario Average (%) = (V + I + F) / 3</t>
   </si>
   <si>
-    <t>(0 / 8,739) = 0 * 100 = 0%</t>
-  </si>
-  <si>
-    <t>Volume recovered (%) = 0%</t>
-  </si>
-  <si>
-    <t>(0 / 0) = 0 * 100 = 0%</t>
+    <t>(8,739 / 8,739) = 1 * 100 = 100%</t>
+  </si>
+  <si>
+    <t>Volume recovered (%) = 100%</t>
+  </si>
+  <si>
+    <t>(87 / 8,739) = 0.01 * 100 = 1%</t>
+  </si>
+  <si>
+    <t>File Integrity (%) = 1%</t>
+  </si>
+  <si>
+    <t>(988 / 8,739) = 0.11 * 100 = 11%</t>
+  </si>
+  <si>
+    <t>Functionality (%) = 11%</t>
+  </si>
+  <si>
+    <t>(100 + 1 + 11) = 112 / 3 = 37.3 %</t>
+  </si>
+  <si>
+    <t>Scenario Average = 37.3%</t>
+  </si>
+  <si>
+    <t>(9,741 / 8,739) = 1.1 * 100 = 110%</t>
+  </si>
+  <si>
+    <t>Volume recovered (%) = 110%</t>
   </si>
   <si>
     <t>File Integrity (%) = 0%</t>
@@ -75,10 +98,34 @@
     <t>Functionality (%) = 0%</t>
   </si>
   <si>
-    <t>(0 + 0 + 0) = 0 / 3 = 0 %</t>
-  </si>
-  <si>
-    <t>Scenario Average = 0%</t>
+    <t>(110 + 0 + 0) = 110 / 3 = 36.67 %</t>
+  </si>
+  <si>
+    <t>Scenario Average = 36.67%</t>
+  </si>
+  <si>
+    <t>(1,120 / 8,739) = 0.13 * 100 = 13%</t>
+  </si>
+  <si>
+    <t>Volume recovered (%) = 13%</t>
+  </si>
+  <si>
+    <t>1,120 / 1,120) = 1 * 100 = 100%</t>
+  </si>
+  <si>
+    <t>Functionality (%) = 100%</t>
+  </si>
+  <si>
+    <t>(13 + 0 + 100) = 113 / 3 = 37.67 %</t>
+  </si>
+  <si>
+    <t>Scenario Average = 37.67%</t>
+  </si>
+  <si>
+    <t>(0 / 1,120) = 0 * 100 = 0%</t>
+  </si>
+  <si>
+    <t>(0 / 9,741) = 0 * 100 = 0%</t>
   </si>
 </sst>
 </file>
@@ -565,7 +612,7 @@
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -576,7 +623,7 @@
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
@@ -599,7 +646,7 @@
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -607,11 +654,311 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EAC7108-323A-4424-802A-F8FC4238A62F}">
+  <dimension ref="B2:I28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E213940-5281-4EE2-9187-20B8BD429D5E}">
+  <dimension ref="B2:I28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="4"/>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added secure erase data for Samsung SSD
</commit_message>
<xml_diff>
--- a/SSD Files/PNY CS900/Secure Erase/Recovery metrics.xlsx
+++ b/SSD Files/PNY CS900/Secure Erase/Recovery metrics.xlsx
@@ -5,17 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\Uni\Dissertation\SSD Files\PNY CS900\Secure Erase\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Documents\Uni\Dissertation\MScProject\SSD Files\PNY CS900\Secure Erase\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12A7E609-08FB-44DB-A69D-48B4481B6824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B9901D-8C24-47EC-84D2-56F9ED82EDB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4720C983-EA5C-4C7A-96E6-6ACFA6986950}"/>
   </bookViews>
   <sheets>
     <sheet name="Autopsy" sheetId="1" r:id="rId1"/>
-    <sheet name="DiskDrill" sheetId="2" r:id="rId2"/>
-    <sheet name="PhotoRec" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Volume</t>
   </si>
@@ -68,12 +66,6 @@
     <t>Volume recovered (%) = 100%</t>
   </si>
   <si>
-    <t>(87 / 8,739) = 0.01 * 100 = 1%</t>
-  </si>
-  <si>
-    <t>File Integrity (%) = 1%</t>
-  </si>
-  <si>
     <t>(988 / 8,739) = 0.11 * 100 = 11%</t>
   </si>
   <si>
@@ -86,46 +78,7 @@
     <t>Scenario Average = 37.3%</t>
   </si>
   <si>
-    <t>(9,741 / 8,739) = 1.1 * 100 = 110%</t>
-  </si>
-  <si>
-    <t>Volume recovered (%) = 110%</t>
-  </si>
-  <si>
-    <t>File Integrity (%) = 0%</t>
-  </si>
-  <si>
-    <t>Functionality (%) = 0%</t>
-  </si>
-  <si>
-    <t>(110 + 0 + 0) = 110 / 3 = 36.67 %</t>
-  </si>
-  <si>
-    <t>Scenario Average = 36.67%</t>
-  </si>
-  <si>
-    <t>(1,120 / 8,739) = 0.13 * 100 = 13%</t>
-  </si>
-  <si>
-    <t>Volume recovered (%) = 13%</t>
-  </si>
-  <si>
-    <t>1,120 / 1,120) = 1 * 100 = 100%</t>
-  </si>
-  <si>
-    <t>Functionality (%) = 100%</t>
-  </si>
-  <si>
-    <t>(13 + 0 + 100) = 113 / 3 = 37.67 %</t>
-  </si>
-  <si>
-    <t>Scenario Average = 37.67%</t>
-  </si>
-  <si>
-    <t>(0 / 1,120) = 0 * 100 = 0%</t>
-  </si>
-  <si>
-    <t>(0 / 9,741) = 0 * 100 = 0%</t>
+    <t>File Integrity (%) = 100%</t>
   </si>
 </sst>
 </file>
@@ -573,7 +526,7 @@
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
       <c r="C12" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -584,7 +537,7 @@
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
@@ -612,7 +565,7 @@
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -623,7 +576,7 @@
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
@@ -646,7 +599,7 @@
     <row r="26" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B26" s="2"/>
       <c r="C26" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -654,311 +607,11 @@
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EAC7108-323A-4424-802A-F8FC4238A62F}">
-  <dimension ref="B2:I28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="4"/>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="2"/>
-      <c r="C26" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E213940-5281-4EE2-9187-20B8BD429D5E}">
-  <dimension ref="B2:I28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B23" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B24" s="4"/>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B25" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B26" s="2"/>
-      <c r="C26" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B28" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>